<commit_message>
Add day3 notebook with data analysis and visualization using pandas
</commit_message>
<xml_diff>
--- a/pandas_crash/GENAIroadmap.xlsx
+++ b/pandas_crash/GENAIroadmap.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GenAI-Portfolio-Yashveer\pandas_crash\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CB1517D-F81B-4190-A6B4-E39700B03F79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A058903-BB5F-4FAE-A7C0-F1322B10E7D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="562" activeTab="1" xr2:uid="{366CEC1A-E31A-4A2D-8F1C-3CAFA0551B2E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="562" xr2:uid="{366CEC1A-E31A-4A2D-8F1C-3CAFA0551B2E}"/>
   </bookViews>
   <sheets>
     <sheet name="roadmap" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="737" uniqueCount="291">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="738" uniqueCount="292">
   <si>
     <t>Section</t>
   </si>
@@ -894,13 +894,16 @@
   </si>
   <si>
     <t>Anthropic Developer Docs</t>
+  </si>
+  <si>
+    <t>Tokenization and Basic Terminologies</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1038,6 +1041,11 @@
     <font>
       <sz val="10"/>
       <color rgb="FF434343"/>
+      <name val="Roboto"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color theme="1"/>
       <name val="Roboto"/>
     </font>
   </fonts>
@@ -1559,7 +1567,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
@@ -1597,6 +1605,7 @@
     <xf numFmtId="0" fontId="18" fillId="33" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -2405,6 +2414,9 @@
       <c r="A38" t="s">
         <v>44</v>
       </c>
+      <c r="B38" s="13" t="s">
+        <v>291</v>
+      </c>
       <c r="C38" t="s">
         <v>9</v>
       </c>

</xml_diff>